<commit_message>
wip(api): phase 5 M3c step 2, sheet formats memory, column mapper, compact matcher, batched catalog writes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/test/fixtures/sheets/precios-multiples-diciembre.xlsx
+++ b/apps/api/test/fixtures/sheets/precios-multiples-diciembre.xlsx
@@ -434,15 +434,15 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SELLADORES</v>
+        <v>SEGURIDAD</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SEL-280</v>
+        <v>CAN-040</v>
       </c>
       <c r="B6" t="str">
-        <v>Silicona transparente 280ml</v>
+        <v>Candado bronce 40mm</v>
       </c>
       <c r="C6" t="str">
         <v>unidad</v>
@@ -462,10 +462,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SEL-500</v>
+        <v>CER-001</v>
       </c>
       <c r="B7" t="str">
-        <v>Sellador acrílico 500g</v>
+        <v>Cerradura de embutir</v>
       </c>
       <c r="C7" t="str">
         <v>unidad</v>
@@ -485,15 +485,15 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>PINTURERÍA</v>
+        <v>HERRAJES</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PIN-023</v>
+        <v>BIS-003</v>
       </c>
       <c r="B9" t="str">
-        <v>Rodillo lana 23cm</v>
+        <v>Bisagra 3 pulgadas</v>
       </c>
       <c r="C9" t="str">
         <v>unidad</v>
@@ -513,13 +513,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>PIN-002</v>
+        <v>TAR-008</v>
       </c>
       <c r="B10" t="str">
-        <v>Pincel 2 pulgadas</v>
+        <v>Tarugo 8mm x100</v>
       </c>
       <c r="C10" t="str">
-        <v>unidad</v>
+        <v>caja</v>
       </c>
       <c r="D10">
         <v>122.95</v>
@@ -536,13 +536,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>LIJ-220</v>
+        <v>PEG-250</v>
       </c>
       <c r="B11" t="str">
-        <v>Lija al agua grano 220</v>
+        <v>Pegamento de contacto 250ml</v>
       </c>
       <c r="C11" t="str">
-        <v>pliego</v>
+        <v>lata</v>
       </c>
       <c r="D11">
         <v>36.07</v>
@@ -559,18 +559,18 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ABRASIVOS</v>
+        <v>ELECTRICIDAD</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>DIS-115</v>
+        <v>CIN-020</v>
       </c>
       <c r="B13" t="str">
-        <v>Disco de corte 115mm</v>
+        <v>Cinta aisladora 20m</v>
       </c>
       <c r="C13" t="str">
-        <v>unidad</v>
+        <v>rollo</v>
       </c>
       <c r="D13">
         <v>81.97</v>
@@ -587,13 +587,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIN-024</v>
+        <v>GUA-00M</v>
       </c>
       <c r="B14" t="str">
-        <v>Cinta de papel 24mm</v>
+        <v>Guante de nitrilo talle M</v>
       </c>
       <c r="C14" t="str">
-        <v>rollo</v>
+        <v>par</v>
       </c>
       <c r="D14">
         <v>94.26</v>
@@ -610,10 +610,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIN-048</v>
+        <v>TAN-002</v>
       </c>
       <c r="B15" t="str">
-        <v>Cinta de papel 48mm</v>
+        <v>Tanza para bordeadora 2mm</v>
       </c>
       <c r="C15" t="str">
         <v>rollo</v>

</xml_diff>